<commit_message>
Set initial stock to 0 for catalog items
</commit_message>
<xml_diff>
--- a/data/catalogo_costos_y_precios_pinto.xlsx
+++ b/data/catalogo_costos_y_precios_pinto.xlsx
@@ -545,7 +545,7 @@
         <v/>
       </c>
       <c r="I2" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -590,7 +590,7 @@
         <v/>
       </c>
       <c r="I3" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -635,7 +635,7 @@
         <v/>
       </c>
       <c r="I4" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -680,7 +680,7 @@
         <v/>
       </c>
       <c r="I5" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -725,7 +725,7 @@
         <v/>
       </c>
       <c r="I6" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -770,7 +770,7 @@
         <v/>
       </c>
       <c r="I7" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -815,7 +815,7 @@
         <v/>
       </c>
       <c r="I8" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -860,7 +860,7 @@
         <v/>
       </c>
       <c r="I9" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -905,7 +905,7 @@
         <v/>
       </c>
       <c r="I10" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -950,7 +950,7 @@
         <v/>
       </c>
       <c r="I11" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -995,7 +995,7 @@
         <v/>
       </c>
       <c r="I12" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
@@ -1040,7 +1040,7 @@
         <v/>
       </c>
       <c r="I13" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -1085,7 +1085,7 @@
         <v/>
       </c>
       <c r="I14" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
@@ -1130,7 +1130,7 @@
         <v/>
       </c>
       <c r="I15" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
@@ -1175,7 +1175,7 @@
         <v/>
       </c>
       <c r="I16" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
@@ -1220,7 +1220,7 @@
         <v/>
       </c>
       <c r="I17" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
@@ -1265,7 +1265,7 @@
         <v/>
       </c>
       <c r="I18" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
@@ -1310,7 +1310,7 @@
         <v/>
       </c>
       <c r="I19" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
@@ -1355,7 +1355,7 @@
         <v/>
       </c>
       <c r="I20" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
@@ -1400,7 +1400,7 @@
         <v/>
       </c>
       <c r="I21" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
@@ -1445,7 +1445,7 @@
         <v/>
       </c>
       <c r="I22" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
@@ -1490,7 +1490,7 @@
         <v/>
       </c>
       <c r="I23" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
@@ -1535,7 +1535,7 @@
         <v/>
       </c>
       <c r="I24" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
@@ -1580,7 +1580,7 @@
         <v/>
       </c>
       <c r="I25" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
@@ -1625,7 +1625,7 @@
         <v/>
       </c>
       <c r="I26" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
@@ -1670,7 +1670,7 @@
         <v/>
       </c>
       <c r="I27" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
@@ -1715,7 +1715,7 @@
         <v/>
       </c>
       <c r="I28" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
@@ -1760,7 +1760,7 @@
         <v/>
       </c>
       <c r="I29" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
@@ -1805,7 +1805,7 @@
         <v/>
       </c>
       <c r="I30" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
@@ -1850,7 +1850,7 @@
         <v/>
       </c>
       <c r="I31" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
@@ -1895,7 +1895,7 @@
         <v/>
       </c>
       <c r="I32" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
@@ -1940,7 +1940,7 @@
         <v/>
       </c>
       <c r="I33" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J33" t="inlineStr">
         <is>
@@ -1985,7 +1985,7 @@
         <v/>
       </c>
       <c r="I34" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J34" t="inlineStr">
         <is>
@@ -2030,7 +2030,7 @@
         <v/>
       </c>
       <c r="I35" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J35" t="inlineStr">
         <is>
@@ -2075,7 +2075,7 @@
         <v/>
       </c>
       <c r="I36" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
@@ -2120,7 +2120,7 @@
         <v/>
       </c>
       <c r="I37" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
@@ -2165,7 +2165,7 @@
         <v/>
       </c>
       <c r="I38" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J38" t="inlineStr">
         <is>
@@ -2210,7 +2210,7 @@
         <v/>
       </c>
       <c r="I39" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J39" t="inlineStr">
         <is>
@@ -2255,7 +2255,7 @@
         <v/>
       </c>
       <c r="I40" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J40" t="inlineStr">
         <is>
@@ -2300,7 +2300,7 @@
         <v/>
       </c>
       <c r="I41" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J41" t="inlineStr">
         <is>
@@ -2345,7 +2345,7 @@
         <v/>
       </c>
       <c r="I42" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J42" t="inlineStr">
         <is>
@@ -2390,7 +2390,7 @@
         <v/>
       </c>
       <c r="I43" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J43" t="inlineStr">
         <is>
@@ -2435,7 +2435,7 @@
         <v/>
       </c>
       <c r="I44" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J44" t="inlineStr">
         <is>
@@ -2480,7 +2480,7 @@
         <v/>
       </c>
       <c r="I45" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J45" t="inlineStr">
         <is>
@@ -2525,7 +2525,7 @@
         <v/>
       </c>
       <c r="I46" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J46" t="inlineStr">
         <is>
@@ -2570,7 +2570,7 @@
         <v/>
       </c>
       <c r="I47" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J47" t="inlineStr">
         <is>
@@ -2615,7 +2615,7 @@
         <v/>
       </c>
       <c r="I48" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J48" t="inlineStr">
         <is>
@@ -2660,7 +2660,7 @@
         <v/>
       </c>
       <c r="I49" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J49" t="inlineStr">
         <is>
@@ -2705,7 +2705,7 @@
         <v/>
       </c>
       <c r="I50" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J50" t="inlineStr">
         <is>
@@ -2750,7 +2750,7 @@
         <v/>
       </c>
       <c r="I51" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J51" t="inlineStr">
         <is>
@@ -2795,7 +2795,7 @@
         <v/>
       </c>
       <c r="I52" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J52" t="inlineStr">
         <is>
@@ -2840,7 +2840,7 @@
         <v/>
       </c>
       <c r="I53" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J53" t="inlineStr">
         <is>
@@ -2885,7 +2885,7 @@
         <v/>
       </c>
       <c r="I54" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J54" t="inlineStr">
         <is>
@@ -2930,7 +2930,7 @@
         <v/>
       </c>
       <c r="I55" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J55" t="inlineStr">
         <is>

</xml_diff>